<commit_message>
Update rota Excel file with latest staff data
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TWH Flexi working.xlsx
+++ b/TWH Flexi working.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\MTWHome\Users_g\gwhite\Appsense\Redirected\Desktop\test book flexi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8786137F-3160-4C19-8A4F-9912C4638D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{8786137F-3160-4C19-8A4F-9912C4638D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF09C3F9-D6D8-466F-B6B8-9E8D89BA375D}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-1344" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,6 +39,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Georgina WHITE</author>
+    <author>WHITE, Georgina (MAIDSTONE AND TUNBRIDGE WELLS NHS TRUST)</author>
   </authors>
   <commentList>
     <comment ref="D4" authorId="0" shapeId="0" xr:uid="{29A1847C-F8C3-43C3-9ADB-676431ED3280}">
@@ -915,23 +916,18 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Georgina WHITE:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-x3 LD's </t>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Georgina WHITE:
+x3 LD's 
+W1 - Mon, Thu, Fri
+W2 - Thu, Fri, Sat
+W3 - Mon, Thu, Fri
+W4 - Thu, Fri, Sun</t>
         </r>
       </text>
     </comment>
@@ -1477,7 +1473,22 @@
         </r>
       </text>
     </comment>
-    <comment ref="D70" authorId="0" shapeId="0" xr:uid="{5684E87D-9A98-4973-8EEA-BCAA398B5BA9}">
+    <comment ref="D69" authorId="1" shapeId="0" xr:uid="{A71F6068-ECAD-4DC8-89C5-553C2B284426}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>WHITE, Georgina (MAIDSTONE AND TUNBRIDGE WELLS NHS TRUST):
+NO nights unless absolutely necessary.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{5684E87D-9A98-4973-8EEA-BCAA398B5BA9}">
       <text>
         <r>
           <rPr>
@@ -1502,7 +1513,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{4620A54D-37BD-4D15-915A-C7C58754318F}">
+    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{4620A54D-37BD-4D15-915A-C7C58754318F}">
       <text>
         <r>
           <rPr>
@@ -1526,7 +1537,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{AF693A44-FC89-4B81-8DC7-EC5FB6EEF65E}">
+    <comment ref="D73" authorId="0" shapeId="0" xr:uid="{AF693A44-FC89-4B81-8DC7-EC5FB6EEF65E}">
       <text>
         <r>
           <rPr>
@@ -1550,7 +1561,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D73" authorId="0" shapeId="0" xr:uid="{5BB62537-912E-4BFD-B3D0-93157AAC1A19}">
+    <comment ref="D74" authorId="0" shapeId="0" xr:uid="{5BB62537-912E-4BFD-B3D0-93157AAC1A19}">
       <text>
         <r>
           <rPr>
@@ -1574,7 +1585,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D74" authorId="0" shapeId="0" xr:uid="{761D5AC6-A973-4EB7-9A0C-0DDA1556A1F9}">
+    <comment ref="D75" authorId="0" shapeId="0" xr:uid="{761D5AC6-A973-4EB7-9A0C-0DDA1556A1F9}">
       <text>
         <r>
           <rPr>
@@ -1598,7 +1609,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D75" authorId="0" shapeId="0" xr:uid="{2974B038-8440-4383-9CE5-43197AE32AE6}">
+    <comment ref="D76" authorId="0" shapeId="0" xr:uid="{2974B038-8440-4383-9CE5-43197AE32AE6}">
       <text>
         <r>
           <rPr>
@@ -1627,7 +1638,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2035" uniqueCount="134">
   <si>
     <t>Band</t>
   </si>
@@ -1719,6 +1730,9 @@
     <t xml:space="preserve">Laura Lewis </t>
   </si>
   <si>
+    <t>wants to reduce hrs</t>
+  </si>
+  <si>
     <t>Ana Sofia Teixeira</t>
   </si>
   <si>
@@ -1728,15 +1742,12 @@
     <t>SET WKD 2 -Mon D, Wed D,  NIGHTS Fri - Sun (w/c 04/09/23), following week  Wed - D, Thu D &amp; Fri D</t>
   </si>
   <si>
-    <t>Corina Oliveira</t>
+    <t>Corrine O'Donnovan</t>
   </si>
   <si>
     <t>E</t>
   </si>
   <si>
-    <t>Corrine O'Donnovan</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
@@ -1758,6 +1769,9 @@
     <t>Nahida Azim</t>
   </si>
   <si>
+    <t>reducing hrs agreed</t>
+  </si>
+  <si>
     <t>Santhosh Thomas</t>
   </si>
   <si>
@@ -1767,6 +1781,9 @@
     <t>Gemma Olive</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>Paulo Silva</t>
   </si>
   <si>
@@ -1809,6 +1826,24 @@
     <t>OFF</t>
   </si>
   <si>
+    <t>Rebecca Edwards</t>
+  </si>
+  <si>
+    <t>Temi Itogbe</t>
+  </si>
+  <si>
+    <t>to start 8th June 2026</t>
+  </si>
+  <si>
+    <t>D or LD</t>
+  </si>
+  <si>
+    <t>LD or D</t>
+  </si>
+  <si>
+    <t>Daniel Pateman</t>
+  </si>
+  <si>
     <t>Charles Okonkwo</t>
   </si>
   <si>
@@ -1818,196 +1853,10 @@
     <t>Ashly Johnson</t>
   </si>
   <si>
-    <t>8-14.30</t>
-  </si>
-  <si>
-    <t>Effie Maurice</t>
-  </si>
-  <si>
-    <t>Jaima Jose</t>
-  </si>
-  <si>
-    <t>Maria Flack</t>
-  </si>
-  <si>
-    <t>MONTH 1</t>
-  </si>
-  <si>
-    <t>MONTH 2</t>
-  </si>
-  <si>
-    <t>Megan Sugars</t>
-  </si>
-  <si>
-    <t>Neethu Varughese</t>
-  </si>
-  <si>
-    <t>          37.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neethu Benny </t>
-  </si>
-  <si>
-    <t>Abhila Joseph</t>
-  </si>
-  <si>
-    <t>Nilo Agduyeng</t>
-  </si>
-  <si>
-    <t>Mildred Mutongi</t>
-  </si>
-  <si>
-    <t>Bianca Moreno</t>
-  </si>
-  <si>
-    <t>Rebecca Edwards</t>
-  </si>
-  <si>
-    <t>Roan Realino</t>
-  </si>
-  <si>
-    <t>Subha Sabu Merin</t>
-  </si>
-  <si>
-    <t>Sony George</t>
-  </si>
-  <si>
-    <t>Jyothi Choorakunnel</t>
-  </si>
-  <si>
-    <t>Joffy John</t>
-  </si>
-  <si>
-    <t>Vinu Varghese</t>
-  </si>
-  <si>
-    <t>Aiswarya Balachandran</t>
-  </si>
-  <si>
-    <t>Aug.25</t>
-  </si>
-  <si>
-    <t>Dipalben Patel</t>
-  </si>
-  <si>
-    <t>Sonia Mechergui</t>
-  </si>
-  <si>
-    <t>Aseel Newcombe</t>
-  </si>
-  <si>
-    <t>Mohammad Komeili</t>
-  </si>
-  <si>
-    <t>any shift</t>
-  </si>
-  <si>
-    <t>Chris Ryan</t>
-  </si>
-  <si>
-    <t>06:00-15:30</t>
-  </si>
-  <si>
-    <t>06:00-16:00</t>
-  </si>
-  <si>
-    <t>Kiko Dias</t>
-  </si>
-  <si>
-    <t>Claudio Vieira</t>
-  </si>
-  <si>
-    <t>Daniel Asbury</t>
-  </si>
-  <si>
-    <t> LD</t>
-  </si>
-  <si>
-    <t>Jane Fox</t>
-  </si>
-  <si>
-    <t>Chloe Jennings</t>
-  </si>
-  <si>
-    <t>E(8-14)</t>
-  </si>
-  <si>
-    <t>Jasmine Thompson</t>
-  </si>
-  <si>
-    <t>Cazeene Marshall</t>
-  </si>
-  <si>
-    <t>Roxanne Yarwood</t>
-  </si>
-  <si>
-    <t>NO nights any shifts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joann Barnes </t>
-  </si>
-  <si>
-    <t> D</t>
-  </si>
-  <si>
-    <t>Denis Cotofrea</t>
-  </si>
-  <si>
-    <t>D/O</t>
-  </si>
-  <si>
-    <t>Urszula Kowalska</t>
-  </si>
-  <si>
-    <t>Suneel Kanakatla</t>
-  </si>
-  <si>
-    <t>Loveth Nnadi</t>
-  </si>
-  <si>
-    <t>Chloe Prenter</t>
-  </si>
-  <si>
-    <t>08-1430</t>
-  </si>
-  <si>
-    <t>check shift pattern</t>
-  </si>
-  <si>
-    <t>any shifts</t>
-  </si>
-  <si>
-    <t>REDUCED HOURS</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>review flexi</t>
-  </si>
-  <si>
-    <t>Daniel Pateman</t>
-  </si>
-  <si>
-    <t>to start check note</t>
-  </si>
-  <si>
-    <t>Temi Itogbe</t>
-  </si>
-  <si>
-    <t>D or LD</t>
-  </si>
-  <si>
-    <t>LD or D</t>
+    <t>to start July 2026</t>
   </si>
   <si>
     <t>DorLDR</t>
-  </si>
-  <si>
-    <t>to start July 2026</t>
-  </si>
-  <si>
-    <t>to start 11 May 2026</t>
   </si>
   <si>
     <r>
@@ -2025,26 +1874,191 @@
     </r>
   </si>
   <si>
-    <t>to start 8th June 2026</t>
-  </si>
-  <si>
-    <t>reducing hrs agreed</t>
-  </si>
-  <si>
-    <t>wants to reduce hrs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">check pattern? </t>
+    <t>to start 11 May 2026</t>
+  </si>
+  <si>
+    <t>08-1430</t>
+  </si>
+  <si>
+    <t>8-14.30</t>
+  </si>
+  <si>
+    <t>Effie Maurice</t>
+  </si>
+  <si>
+    <t>Jaima Jose</t>
+  </si>
+  <si>
+    <t>Maria Flack</t>
+  </si>
+  <si>
+    <t>MONTH 1</t>
+  </si>
+  <si>
+    <t>MONTH 2</t>
+  </si>
+  <si>
+    <t>Megan Sugars</t>
+  </si>
+  <si>
+    <t>Neethu Varughese</t>
+  </si>
+  <si>
+    <t>          37.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neethu Benny </t>
+  </si>
+  <si>
+    <t>Abhila Joseph</t>
+  </si>
+  <si>
+    <t>Nilo Agduyeng</t>
+  </si>
+  <si>
+    <t>Mildred Mutongi</t>
+  </si>
+  <si>
+    <t>Bianca Moreno</t>
+  </si>
+  <si>
+    <t>Roan Realino</t>
+  </si>
+  <si>
+    <t>Subha Sabu Merin</t>
+  </si>
+  <si>
+    <t>Sony George</t>
+  </si>
+  <si>
+    <t>Jyothi Choorakunnel</t>
+  </si>
+  <si>
+    <t>Joffy John</t>
+  </si>
+  <si>
+    <t>Vinu Varghese</t>
+  </si>
+  <si>
+    <t>Aiswarya Balachandran</t>
+  </si>
+  <si>
+    <t>Aug.25</t>
+  </si>
+  <si>
+    <t>Dipalben Patel</t>
+  </si>
+  <si>
+    <t>Sonia Mechergui</t>
+  </si>
+  <si>
+    <t>Aseel Newcombe</t>
+  </si>
+  <si>
+    <t>Mohammad Komeili</t>
+  </si>
+  <si>
+    <t>any shift</t>
+  </si>
+  <si>
+    <t>any shifts</t>
+  </si>
+  <si>
+    <t>Chris Ryan</t>
+  </si>
+  <si>
+    <t>06:00-15:30</t>
+  </si>
+  <si>
+    <t>06:00-16:00</t>
+  </si>
+  <si>
+    <t>Kiko Dias</t>
+  </si>
+  <si>
+    <t>Claudio Vieira</t>
+  </si>
+  <si>
+    <t>Daniel Asbury</t>
+  </si>
+  <si>
+    <t> LD</t>
+  </si>
+  <si>
+    <t>Jane Fox</t>
+  </si>
+  <si>
+    <t>Chloe Jennings</t>
+  </si>
+  <si>
+    <t>E(8-14)</t>
+  </si>
+  <si>
+    <t>Jasmine Thompson</t>
+  </si>
+  <si>
+    <t>Cazeene Marshall</t>
+  </si>
+  <si>
+    <t>Nicola Atkinson</t>
+  </si>
+  <si>
+    <t>to start 8th June 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joann Barnes </t>
+  </si>
+  <si>
+    <t> D</t>
+  </si>
+  <si>
+    <t>Denis Cotofrea</t>
+  </si>
+  <si>
+    <t>D/O</t>
+  </si>
+  <si>
+    <t>Urszula Kowalska</t>
+  </si>
+  <si>
+    <t>Suneel Kanakatla</t>
+  </si>
+  <si>
+    <t>Loveth Nnadi</t>
+  </si>
+  <si>
+    <t>Chloe Prenter</t>
   </si>
   <si>
     <t>Leaving/Left</t>
+  </si>
+  <si>
+    <t>Roxanne Yarwood</t>
+  </si>
+  <si>
+    <t>NO nights any shifts</t>
+  </si>
+  <si>
+    <t>Corina Oliveira</t>
+  </si>
+  <si>
+    <t>review flexi</t>
+  </si>
+  <si>
+    <t>REDUCED HOURS</t>
+  </si>
+  <si>
+    <t>to start check note</t>
+  </si>
+  <si>
+    <t>check shift pattern</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2463,7 +2477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="213">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2695,7 +2709,6 @@
     <xf numFmtId="17" fontId="4" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="4" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -2714,6 +2727,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="17" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="4" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2722,11 +2739,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <mruColors>
-      <color rgb="FFFFFF99"/>
       <color rgb="FFB2B2B2"/>
-      <color rgb="FF99FFCC"/>
       <color rgb="FFFFCCFF"/>
       <color rgb="FF33CCCC"/>
+      <color rgb="FFFFFF99"/>
+      <color rgb="FF99FFCC"/>
       <color rgb="FFFF66FF"/>
       <color rgb="FFFFCCCC"/>
       <color rgb="FFFF99CC"/>
@@ -3062,13 +3079,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP91"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AP92"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.140625" style="18" customWidth="1"/>
     <col min="2" max="2" width="21.28515625" style="109" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" style="201" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" style="18" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="200" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="18" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" style="18" customWidth="1"/>
     <col min="6" max="6" width="11" style="18" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" style="18" customWidth="1"/>
@@ -3102,14 +3119,14 @@
     <col min="39" max="16384" width="8.7109375" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="197" t="s">
+      <c r="C1" s="196" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="15" t="s">
@@ -3218,7 +3235,7 @@
       <c r="AM1" s="14"/>
       <c r="AN1" s="14"/>
     </row>
-    <row r="2" spans="1:40" s="186" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" s="186" customFormat="1" ht="14.45" customHeight="1">
       <c r="A2" s="179">
         <v>8</v>
       </c>
@@ -3314,7 +3331,7 @@
       <c r="AM2" s="182"/>
       <c r="AN2" s="182"/>
     </row>
-    <row r="3" spans="1:40" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:40" ht="14.45" customHeight="1">
       <c r="A3" s="19"/>
       <c r="B3" s="20"/>
       <c r="C3" s="21"/>
@@ -3352,7 +3369,7 @@
       <c r="AM3" s="22"/>
       <c r="AN3" s="22"/>
     </row>
-    <row r="4" spans="1:40" s="33" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:40" s="33" customFormat="1" ht="13.9" customHeight="1">
       <c r="A4" s="25">
         <v>7</v>
       </c>
@@ -3467,7 +3484,7 @@
       </c>
       <c r="AM4" s="32"/>
     </row>
-    <row r="5" spans="1:40" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:40" s="142" customFormat="1">
       <c r="A5" s="132">
         <v>7</v>
       </c>
@@ -3580,7 +3597,7 @@
       <c r="AL5" s="137"/>
       <c r="AM5" s="145"/>
     </row>
-    <row r="6" spans="1:40" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:40" s="142" customFormat="1">
       <c r="A6" s="134">
         <v>7</v>
       </c>
@@ -3695,7 +3712,7 @@
       </c>
       <c r="AM6" s="145"/>
     </row>
-    <row r="7" spans="1:40" s="130" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:40" s="130" customFormat="1">
       <c r="A7" s="132">
         <v>7</v>
       </c>
@@ -3706,7 +3723,7 @@
         <v>45748</v>
       </c>
       <c r="D7" s="125" t="s">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="E7" s="130" t="s">
         <v>4</v>
@@ -3776,12 +3793,12 @@
       </c>
       <c r="AM7" s="129"/>
     </row>
-    <row r="8" spans="1:40" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:40" s="142" customFormat="1">
       <c r="A8" s="134">
         <v>7</v>
       </c>
       <c r="B8" s="135" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="136">
         <v>44774</v>
@@ -3891,12 +3908,12 @@
       </c>
       <c r="AM8" s="145"/>
     </row>
-    <row r="9" spans="1:40" s="33" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:40" s="33" customFormat="1">
       <c r="A9" s="25">
         <v>7</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="27">
         <v>45870</v>
@@ -4002,11 +4019,11 @@
         <v>37.5</v>
       </c>
       <c r="AL9" s="28" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AM9" s="32"/>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:40">
       <c r="A10" s="34"/>
       <c r="B10" s="35"/>
       <c r="C10" s="36"/>
@@ -4043,12 +4060,12 @@
       <c r="AL10" s="37"/>
       <c r="AM10" s="22"/>
     </row>
-    <row r="11" spans="1:40" s="142" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:40" s="142" customFormat="1" ht="13.9" customHeight="1">
       <c r="A11" s="134">
         <v>6</v>
       </c>
       <c r="B11" s="135" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="136">
         <v>45261</v>
@@ -4061,13 +4078,13 @@
         <v>21</v>
       </c>
       <c r="G11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H11" s="138" t="s">
         <v>18</v>
       </c>
       <c r="I11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J11" s="138" t="s">
         <v>21</v>
@@ -4085,13 +4102,13 @@
         <v>21</v>
       </c>
       <c r="O11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P11" s="138" t="s">
         <v>18</v>
       </c>
       <c r="Q11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R11" s="138" t="s">
         <v>21</v>
@@ -4105,13 +4122,13 @@
         <v>21</v>
       </c>
       <c r="W11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X11" s="138" t="s">
         <v>18</v>
       </c>
       <c r="Y11" s="138" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z11" s="138" t="s">
         <v>21</v>
@@ -4140,7 +4157,7 @@
       </c>
       <c r="AM11" s="145"/>
     </row>
-    <row r="12" spans="1:40" s="142" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:40" s="142" customFormat="1" ht="14.45" customHeight="1">
       <c r="A12" s="134">
         <v>6</v>
       </c>
@@ -4211,14 +4228,14 @@
       <c r="AL12" s="137"/>
       <c r="AM12" s="145"/>
     </row>
-    <row r="13" spans="1:40" s="58" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:40" s="58" customFormat="1" ht="17.45" customHeight="1">
       <c r="A13" s="132">
         <v>6</v>
       </c>
       <c r="B13" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="196">
+      <c r="C13" s="195">
         <v>46082</v>
       </c>
       <c r="D13" s="59"/>
@@ -4326,7 +4343,7 @@
       </c>
       <c r="AM13" s="57"/>
     </row>
-    <row r="14" spans="1:40" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:40" s="142" customFormat="1">
       <c r="A14" s="134">
         <v>6</v>
       </c>
@@ -4439,129 +4456,129 @@
       <c r="AL14" s="137"/>
       <c r="AM14" s="145"/>
     </row>
-    <row r="15" spans="1:40" s="130" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="122">
+    <row r="15" spans="1:40" s="58" customFormat="1">
+      <c r="A15" s="132">
         <v>6</v>
       </c>
-      <c r="B15" s="123" t="s">
+      <c r="B15" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="124">
+      <c r="C15" s="52">
         <v>46447</v>
       </c>
-      <c r="D15" s="195" t="s">
-        <v>129</v>
-      </c>
-      <c r="E15" s="130" t="s">
+      <c r="D15" s="212" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="H15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="K15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="125" t="s">
-        <v>18</v>
-      </c>
-      <c r="M15" s="130" t="s">
+      <c r="F15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="N15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="O15" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="S15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="T15" s="125" t="s">
-        <v>18</v>
-      </c>
-      <c r="U15" s="130" t="s">
+      <c r="N15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="O15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="P15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="S15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="T15" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="U15" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="V15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="W15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="X15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA15" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB15" s="125" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC15" s="130" t="s">
+      <c r="V15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="W15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="X15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB15" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC15" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="AD15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="AE15" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AF15" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG15" s="126" t="s">
-        <v>18</v>
-      </c>
-      <c r="AH15" s="125" t="s">
-        <v>21</v>
-      </c>
-      <c r="AI15" s="127" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ15" s="128" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK15" s="126">
+      <c r="AD15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF15" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG15" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH15" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI15" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ15" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK15" s="54">
         <v>28.5</v>
       </c>
-      <c r="AL15" s="125" t="s">
+      <c r="AL15" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AM15" s="129"/>
+      <c r="AM15" s="57"/>
     </row>
-    <row r="16" spans="1:40" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:40" s="142" customFormat="1">
       <c r="A16" s="134">
         <v>6</v>
       </c>
       <c r="B16" s="135" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="136">
         <v>44593</v>
@@ -4669,12 +4686,12 @@
       <c r="AL16" s="137"/>
       <c r="AM16" s="145"/>
     </row>
-    <row r="17" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" s="142" customFormat="1">
       <c r="A17" s="134">
         <v>6</v>
       </c>
       <c r="B17" s="135" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" s="136">
         <v>45901</v>
@@ -4782,18 +4799,18 @@
       <c r="AL17" s="137"/>
       <c r="AM17" s="145"/>
     </row>
-    <row r="18" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" s="142" customFormat="1">
       <c r="A18" s="134">
         <v>6</v>
       </c>
       <c r="B18" s="135" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C18" s="136">
         <v>45809</v>
       </c>
       <c r="D18" s="177" t="s">
-        <v>117</v>
+        <v>47</v>
       </c>
       <c r="E18" s="142" t="s">
         <v>4</v>
@@ -4869,12 +4886,12 @@
       <c r="AL18" s="137"/>
       <c r="AM18" s="145"/>
     </row>
-    <row r="19" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:39" s="58" customFormat="1">
       <c r="A19" s="50">
         <v>6</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C19" s="52">
         <v>46113</v>
@@ -4978,16 +4995,16 @@
       </c>
       <c r="AK19" s="54"/>
       <c r="AL19" s="53" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AM19" s="57"/>
     </row>
-    <row r="20" spans="1:39" s="58" customFormat="1" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:39" s="58" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A20" s="50">
         <v>6</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C20" s="52">
         <v>45901</v>
@@ -5055,16 +5072,16 @@
         <v>37.5</v>
       </c>
       <c r="AL20" s="53" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AM20" s="57"/>
     </row>
-    <row r="21" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" s="142" customFormat="1">
       <c r="A21" s="132">
         <v>6</v>
       </c>
       <c r="B21" s="135" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C21" s="136"/>
       <c r="D21" s="137"/>
@@ -5114,12 +5131,12 @@
       <c r="AL21" s="137"/>
       <c r="AM21" s="145"/>
     </row>
-    <row r="22" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:39" s="58" customFormat="1">
       <c r="A22" s="50">
         <v>6</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C22" s="52">
         <v>45748</v>
@@ -5183,14 +5200,14 @@
       <c r="AL22" s="53"/>
       <c r="AM22" s="57"/>
     </row>
-    <row r="23" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" s="142" customFormat="1">
       <c r="A23" s="187">
         <v>6</v>
       </c>
       <c r="B23" s="188" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="198"/>
+        <v>54</v>
+      </c>
+      <c r="C23" s="197"/>
       <c r="D23" s="141"/>
       <c r="E23" s="142" t="s">
         <v>4</v>
@@ -5293,33 +5310,33 @@
       </c>
       <c r="AL23" s="141"/>
     </row>
-    <row r="24" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" s="58" customFormat="1">
       <c r="A24" s="133">
         <v>6</v>
       </c>
-      <c r="B24" s="204" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="205"/>
+      <c r="B24" s="203" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="204"/>
       <c r="E24" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="F24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" s="206" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="I24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="J24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="K24" s="206" t="s">
+      <c r="F24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="205" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="205" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="J24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="K24" s="205" t="s">
         <v>27</v>
       </c>
       <c r="L24" s="58" t="s">
@@ -5328,22 +5345,22 @@
       <c r="M24" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="N24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="O24" s="206" t="s">
-        <v>21</v>
-      </c>
-      <c r="P24" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q24" s="206" t="s">
-        <v>21</v>
-      </c>
-      <c r="R24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="S24" s="206" t="s">
+      <c r="N24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="O24" s="205" t="s">
+        <v>21</v>
+      </c>
+      <c r="P24" s="205" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q24" s="205" t="s">
+        <v>21</v>
+      </c>
+      <c r="R24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="S24" s="205" t="s">
         <v>18</v>
       </c>
       <c r="T24" s="58" t="s">
@@ -5352,22 +5369,22 @@
       <c r="U24" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="V24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="W24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="X24" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z24" s="206" t="s">
+      <c r="V24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="W24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="X24" s="205" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z24" s="205" t="s">
         <v>36</v>
       </c>
-      <c r="AA24" s="206" t="s">
+      <c r="AA24" s="205" t="s">
         <v>36</v>
       </c>
       <c r="AB24" s="58" t="s">
@@ -5376,39 +5393,39 @@
       <c r="AC24" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="AD24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="AE24" s="206" t="s">
-        <v>18</v>
-      </c>
-      <c r="AF24" s="206" t="s">
-        <v>27</v>
-      </c>
-      <c r="AG24" s="206" t="s">
+      <c r="AD24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE24" s="205" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF24" s="205" t="s">
+        <v>27</v>
+      </c>
+      <c r="AG24" s="205" t="s">
         <v>21</v>
       </c>
       <c r="AH24" s="58" t="s">
-        <v>34</v>
-      </c>
-      <c r="AI24" s="207" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ24" s="208" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK24" s="209" t="s">
+        <v>35</v>
+      </c>
+      <c r="AI24" s="206" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ24" s="207" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK24" s="208" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:39" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="202">
+    <row r="25" spans="1:39" s="68" customFormat="1">
+      <c r="A25" s="201">
         <v>6</v>
       </c>
       <c r="B25" s="69" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="199">
+        <v>56</v>
+      </c>
+      <c r="C25" s="198">
         <v>45772</v>
       </c>
       <c r="D25" s="70"/>
@@ -5452,7 +5469,7 @@
         <v>18</v>
       </c>
       <c r="R25" s="68" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S25" s="68" t="s">
         <v>18</v>
@@ -5516,12 +5533,12 @@
       </c>
       <c r="AM25" s="72"/>
     </row>
-    <row r="26" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" s="58" customFormat="1">
       <c r="A26" s="50">
         <v>6</v>
       </c>
       <c r="B26" s="51" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C26" s="52">
         <v>45809</v>
@@ -5631,12 +5648,12 @@
       </c>
       <c r="AM26" s="57"/>
     </row>
-    <row r="27" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" s="58" customFormat="1">
       <c r="A27" s="62">
         <v>6</v>
       </c>
       <c r="B27" s="63" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C27" s="2">
         <v>46296</v>
@@ -5724,12 +5741,12 @@
       <c r="AL27" s="53"/>
       <c r="AM27" s="57"/>
     </row>
-    <row r="28" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:39" s="58" customFormat="1">
       <c r="A28" s="62">
         <v>6</v>
       </c>
       <c r="B28" s="63" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C28" s="2">
         <v>46291</v>
@@ -5836,12 +5853,12 @@
       <c r="AL28" s="53"/>
       <c r="AM28" s="57"/>
     </row>
-    <row r="29" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:39" s="58" customFormat="1">
       <c r="A29" s="62">
         <v>6</v>
       </c>
       <c r="B29" s="63" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C29" s="2">
         <v>46296</v>
@@ -5862,13 +5879,13 @@
         <v>21</v>
       </c>
       <c r="J29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L29" s="65" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="M29" s="58" t="s">
         <v>12</v>
@@ -5886,13 +5903,13 @@
         <v>21</v>
       </c>
       <c r="R29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="S29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="T29" s="65" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="U29" s="58" t="s">
         <v>13</v>
@@ -5904,13 +5921,13 @@
         <v>21</v>
       </c>
       <c r="X29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="Y29" s="64" t="s">
         <v>21</v>
       </c>
       <c r="Z29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AA29" s="64" t="s">
         <v>21</v>
@@ -5925,10 +5942,10 @@
         <v>21</v>
       </c>
       <c r="AE29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AF29" s="64" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AG29" s="64" t="s">
         <v>21</v>
@@ -5937,10 +5954,10 @@
         <v>21</v>
       </c>
       <c r="AI29" s="66" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AJ29" s="67" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AK29" s="3" t="s">
         <v>39</v>
@@ -5948,12 +5965,12 @@
       <c r="AL29" s="53"/>
       <c r="AM29" s="57"/>
     </row>
-    <row r="30" spans="1:39" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" s="58" customFormat="1">
       <c r="A30" s="132">
         <v>6</v>
       </c>
       <c r="B30" s="51" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C30" s="52"/>
       <c r="D30" s="53"/>
@@ -6059,10 +6076,10 @@
       <c r="AL30" s="53"/>
       <c r="AM30" s="57"/>
     </row>
-    <row r="31" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39">
       <c r="A31" s="34"/>
       <c r="B31" s="35"/>
-      <c r="C31" s="203"/>
+      <c r="C31" s="202"/>
       <c r="D31" s="22"/>
       <c r="F31" s="38"/>
       <c r="G31" s="38"/>
@@ -6095,18 +6112,18 @@
       <c r="AL31" s="37"/>
       <c r="AM31" s="22"/>
     </row>
-    <row r="32" spans="1:39" s="120" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" s="120" customFormat="1">
       <c r="A32" s="112">
         <v>5</v>
       </c>
       <c r="B32" s="113" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="C32" s="192">
         <v>46327</v>
       </c>
       <c r="D32" s="119" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="F32" s="116" t="s">
         <v>21</v>
@@ -6124,10 +6141,10 @@
         <v>18</v>
       </c>
       <c r="K32" s="116" t="s">
-        <v>122</v>
+        <v>65</v>
       </c>
       <c r="L32" s="115" t="s">
-        <v>123</v>
+        <v>66</v>
       </c>
       <c r="N32" s="116" t="s">
         <v>21</v>
@@ -6198,18 +6215,18 @@
       <c r="AL32" s="115"/>
       <c r="AM32" s="119"/>
     </row>
-    <row r="33" spans="1:39" s="120" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" s="120" customFormat="1">
       <c r="A33" s="112">
         <v>5</v>
       </c>
       <c r="B33" s="113" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
       <c r="C33" s="192">
         <v>46357</v>
       </c>
       <c r="D33" s="119" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="F33" s="116" t="s">
         <v>18</v>
@@ -6301,12 +6318,12 @@
       <c r="AL33" s="115"/>
       <c r="AM33" s="119"/>
     </row>
-    <row r="34" spans="1:39" s="82" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" s="82" customFormat="1" ht="18.600000000000001" customHeight="1">
       <c r="A34" s="73">
         <v>5</v>
       </c>
       <c r="B34" s="74" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C34" s="4">
         <v>46199</v>
@@ -6414,12 +6431,12 @@
       <c r="AL34" s="80"/>
       <c r="AM34" s="81"/>
     </row>
-    <row r="35" spans="1:39" s="142" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" s="142" customFormat="1" ht="18.600000000000001" customHeight="1">
       <c r="A35" s="194">
         <v>5</v>
       </c>
       <c r="B35" s="135" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C35" s="136">
         <v>45352</v>
@@ -6527,18 +6544,18 @@
       <c r="AL35" s="137"/>
       <c r="AM35" s="145"/>
     </row>
-    <row r="36" spans="1:39" s="120" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" s="120" customFormat="1" ht="18.600000000000001" customHeight="1">
       <c r="A36" s="112">
         <v>5</v>
       </c>
       <c r="B36" s="113" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C36" s="192">
         <v>46388</v>
       </c>
       <c r="D36" s="193" t="s">
-        <v>125</v>
+        <v>71</v>
       </c>
       <c r="E36" s="120" t="s">
         <v>4</v>
@@ -6592,7 +6609,7 @@
         <v>13</v>
       </c>
       <c r="V36" s="116" t="s">
-        <v>124</v>
+        <v>72</v>
       </c>
       <c r="W36" s="116" t="s">
         <v>18</v>
@@ -6644,18 +6661,18 @@
       </c>
       <c r="AM36" s="119"/>
     </row>
-    <row r="37" spans="1:39" s="120" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" s="120" customFormat="1" ht="18.600000000000001" customHeight="1">
       <c r="A37" s="112">
         <v>5</v>
       </c>
       <c r="B37" s="113" t="s">
-        <v>127</v>
+        <v>73</v>
       </c>
       <c r="C37" s="114">
         <v>46327</v>
       </c>
       <c r="D37" s="115" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="E37" s="120" t="s">
         <v>4</v>
@@ -6688,7 +6705,7 @@
         <v>18</v>
       </c>
       <c r="O37" s="116" t="s">
-        <v>113</v>
+        <v>75</v>
       </c>
       <c r="P37" s="116" t="s">
         <v>27</v>
@@ -6697,7 +6714,7 @@
         <v>28</v>
       </c>
       <c r="R37" s="116" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S37" s="116" t="s">
         <v>18</v>
@@ -6736,7 +6753,7 @@
         <v>22</v>
       </c>
       <c r="AE37" s="116" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="AF37" s="116" t="s">
         <v>27</v>
@@ -6745,7 +6762,7 @@
         <v>27</v>
       </c>
       <c r="AH37" s="115" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AI37" s="117" t="s">
         <v>18</v>
@@ -6757,12 +6774,12 @@
       <c r="AL37" s="115"/>
       <c r="AM37" s="119"/>
     </row>
-    <row r="38" spans="1:39" s="82" customFormat="1" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" s="82" customFormat="1" ht="18.600000000000001" customHeight="1">
       <c r="A38" s="132">
         <v>5</v>
       </c>
       <c r="B38" s="84" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C38" s="85">
         <v>44958</v>
@@ -6870,12 +6887,12 @@
       <c r="AL38" s="80"/>
       <c r="AM38" s="81"/>
     </row>
-    <row r="39" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" s="82" customFormat="1">
       <c r="A39" s="83">
         <v>5</v>
       </c>
       <c r="B39" s="84" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C39" s="85">
         <v>46235</v>
@@ -6983,19 +7000,19 @@
       <c r="AL39" s="80"/>
       <c r="AM39" s="81"/>
     </row>
-    <row r="40" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" s="82" customFormat="1">
       <c r="A40" s="132">
         <v>5</v>
       </c>
       <c r="B40" s="84" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C40" s="85">
         <v>45931</v>
       </c>
       <c r="D40" s="80"/>
       <c r="E40" s="82" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="F40" s="86" t="s">
         <v>36</v>
@@ -7049,13 +7066,13 @@
         <v>18</v>
       </c>
       <c r="W40" s="86" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X40" s="86" t="s">
         <v>18</v>
       </c>
       <c r="Y40" s="86" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z40" s="86" t="s">
         <v>18</v>
@@ -7098,13 +7115,13 @@
       </c>
       <c r="AM40" s="81"/>
     </row>
-    <row r="41" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" s="82" customFormat="1">
       <c r="A41" s="83"/>
       <c r="B41" s="84"/>
       <c r="C41" s="85"/>
       <c r="D41" s="80"/>
       <c r="E41" s="82" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="F41" s="86" t="s">
         <v>36</v>
@@ -7164,7 +7181,7 @@
         <v>18</v>
       </c>
       <c r="Y41" s="86" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z41" s="86" t="s">
         <v>18</v>
@@ -7205,12 +7222,12 @@
       <c r="AL41" s="80"/>
       <c r="AM41" s="81"/>
     </row>
-    <row r="42" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:39" s="82" customFormat="1">
       <c r="A42" s="132">
         <v>5</v>
       </c>
       <c r="B42" s="84" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C42" s="85">
         <v>46082</v>
@@ -7318,12 +7335,12 @@
       <c r="AL42" s="80"/>
       <c r="AM42" s="81"/>
     </row>
-    <row r="43" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:39" s="82" customFormat="1">
       <c r="A43" s="83">
         <v>5</v>
       </c>
       <c r="B43" s="84" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C43" s="85">
         <v>45870</v>
@@ -7426,17 +7443,17 @@
         <v>18</v>
       </c>
       <c r="AK43" s="86" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="AL43" s="80"/>
       <c r="AM43" s="81"/>
     </row>
-    <row r="44" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:39" s="142" customFormat="1">
       <c r="A44" s="134">
         <v>5</v>
       </c>
       <c r="B44" s="135" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="C44" s="136">
         <v>44958</v>
@@ -7500,19 +7517,17 @@
       <c r="AL44" s="137"/>
       <c r="AM44" s="145"/>
     </row>
-    <row r="45" spans="1:39" s="130" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:39" s="130" customFormat="1">
       <c r="A45" s="122">
         <v>5</v>
       </c>
       <c r="B45" s="123" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C45" s="124">
         <v>45597</v>
       </c>
-      <c r="D45" s="125" t="s">
-        <v>131</v>
-      </c>
+      <c r="D45" s="125"/>
       <c r="E45" s="130" t="s">
         <v>4</v>
       </c>
@@ -7615,12 +7630,12 @@
       <c r="AL45" s="125"/>
       <c r="AM45" s="129"/>
     </row>
-    <row r="46" spans="1:39" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:39" s="142" customFormat="1">
       <c r="A46" s="134">
         <v>5</v>
       </c>
       <c r="B46" s="135" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="C46" s="136">
         <v>45170</v>
@@ -7682,12 +7697,12 @@
       <c r="AL46" s="137"/>
       <c r="AM46" s="145"/>
     </row>
-    <row r="47" spans="1:39" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:39" s="82" customFormat="1">
       <c r="A47" s="83">
         <v>5</v>
       </c>
       <c r="B47" s="84" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="C47" s="85">
         <v>45962</v>
@@ -7747,12 +7762,12 @@
       <c r="AL47" s="80"/>
       <c r="AM47" s="81"/>
     </row>
-    <row r="48" spans="1:39" s="82" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:39" s="82" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A48" s="83">
         <v>5</v>
       </c>
       <c r="B48" s="84" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="C48" s="85">
         <v>46204</v>
@@ -7860,12 +7875,12 @@
       <c r="AL48" s="80"/>
       <c r="AM48" s="81"/>
     </row>
-    <row r="49" spans="1:42" s="142" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:42" s="142" customFormat="1" ht="15.75" customHeight="1">
       <c r="A49" s="134">
         <v>5</v>
       </c>
       <c r="B49" s="135" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C49" s="136">
         <v>45901</v>
@@ -7975,12 +7990,12 @@
       </c>
       <c r="AM49" s="145"/>
     </row>
-    <row r="50" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:42" s="82" customFormat="1">
       <c r="A50" s="83">
         <v>5</v>
       </c>
       <c r="B50" s="84" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C50" s="85">
         <v>46054</v>
@@ -8088,12 +8103,12 @@
       <c r="AL50" s="80"/>
       <c r="AM50" s="81"/>
     </row>
-    <row r="51" spans="1:42" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:42" s="142" customFormat="1">
       <c r="A51" s="134">
         <v>5</v>
       </c>
       <c r="B51" s="135" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C51" s="136">
         <v>45597</v>
@@ -8200,12 +8215,12 @@
       </c>
       <c r="AL51" s="141"/>
     </row>
-    <row r="52" spans="1:42" s="82" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:42" s="82" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A52" s="83">
         <v>5</v>
       </c>
       <c r="B52" s="84" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C52" s="85">
         <v>47054</v>
@@ -8272,7 +8287,7 @@
         <v>18</v>
       </c>
       <c r="Y52" s="86" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z52" s="86" t="s">
         <v>36</v>
@@ -8312,12 +8327,12 @@
       </c>
       <c r="AL52" s="77"/>
     </row>
-    <row r="53" spans="1:42" s="82" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:42" s="82" customFormat="1" ht="18" customHeight="1">
       <c r="A53" s="73">
         <v>5</v>
       </c>
       <c r="B53" s="74" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C53" s="90">
         <v>45383</v>
@@ -8425,12 +8440,12 @@
       <c r="AL53" s="80"/>
       <c r="AM53" s="81"/>
     </row>
-    <row r="54" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:42" s="82" customFormat="1">
       <c r="A54" s="73">
         <v>5</v>
       </c>
       <c r="B54" s="74" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C54" s="90">
         <v>45955</v>
@@ -8506,15 +8521,15 @@
       <c r="AL54" s="80"/>
       <c r="AM54" s="81"/>
     </row>
-    <row r="55" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:42" s="82" customFormat="1">
       <c r="A55" s="73">
         <v>5</v>
       </c>
       <c r="B55" s="74" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D55" s="77"/>
       <c r="E55" s="82" t="s">
@@ -8619,12 +8634,12 @@
       <c r="AL55" s="80"/>
       <c r="AM55" s="81"/>
     </row>
-    <row r="56" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:42" s="82" customFormat="1">
       <c r="A56" s="83">
         <v>5</v>
       </c>
       <c r="B56" s="84" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="C56" s="85">
         <v>46266</v>
@@ -8735,12 +8750,12 @@
       <c r="AO56" s="91"/>
       <c r="AP56" s="91"/>
     </row>
-    <row r="57" spans="1:42" s="142" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:42" s="142" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A57" s="134">
         <v>5</v>
       </c>
       <c r="B57" s="135" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C57" s="136"/>
       <c r="D57" s="137"/>
@@ -8844,12 +8859,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="58" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:42" s="82" customFormat="1">
       <c r="A58" s="83">
         <v>5</v>
       </c>
       <c r="B58" s="84" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C58" s="85">
         <v>46321</v>
@@ -8955,12 +8970,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="59" spans="1:42" s="82" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:42" s="82" customFormat="1">
       <c r="A59" s="83">
         <v>5</v>
       </c>
       <c r="B59" s="84" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C59" s="85">
         <v>46291</v>
@@ -8979,7 +8994,7 @@
       <c r="I59" s="86"/>
       <c r="J59" s="86"/>
       <c r="K59" s="86" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="L59" s="80" t="s">
         <v>21</v>
@@ -9036,7 +9051,7 @@
         <v>14</v>
       </c>
       <c r="AD59" s="86" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="AE59" s="86"/>
       <c r="AF59" s="86"/>
@@ -9048,7 +9063,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="60" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:42">
       <c r="A60" s="34"/>
       <c r="B60" s="35"/>
       <c r="C60" s="36"/>
@@ -9083,12 +9098,12 @@
       <c r="AJ60" s="40"/>
       <c r="AK60" s="9"/>
     </row>
-    <row r="61" spans="1:42" s="99" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:42" s="99" customFormat="1">
       <c r="A61" s="92">
         <v>3</v>
       </c>
       <c r="B61" s="93" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="C61" s="100"/>
       <c r="D61" s="95"/>
@@ -9096,19 +9111,19 @@
         <v>4</v>
       </c>
       <c r="F61" s="94" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="G61" s="94" t="s">
         <v>18</v>
       </c>
       <c r="H61" s="94" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="I61" s="94" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="J61" s="94" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="K61" s="94" t="s">
         <v>23</v>
@@ -9154,12 +9169,12 @@
       </c>
       <c r="AM61" s="98"/>
     </row>
-    <row r="62" spans="1:42" s="99" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:42" s="99" customFormat="1">
       <c r="A62" s="92">
         <v>3</v>
       </c>
       <c r="B62" s="93" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="C62" s="100">
         <v>46174</v>
@@ -9267,12 +9282,12 @@
       <c r="AL62" s="95"/>
       <c r="AM62" s="98"/>
     </row>
-    <row r="63" spans="1:42" s="99" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:42" s="99" customFormat="1">
       <c r="A63" s="92">
         <v>3</v>
       </c>
       <c r="B63" s="93" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="C63" s="100">
         <v>46478</v>
@@ -9380,12 +9395,12 @@
       <c r="AL63" s="95"/>
       <c r="AM63" s="98"/>
     </row>
-    <row r="64" spans="1:42" s="99" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:42" s="99" customFormat="1">
       <c r="A64" s="132">
         <v>3</v>
       </c>
       <c r="B64" s="93" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C64" s="100"/>
       <c r="D64" s="95"/>
@@ -9403,7 +9418,7 @@
         <v>23</v>
       </c>
       <c r="J64" s="94" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="K64" s="94"/>
       <c r="L64" s="95" t="s">
@@ -9457,12 +9472,12 @@
       <c r="AL64" s="95"/>
       <c r="AM64" s="98"/>
     </row>
-    <row r="65" spans="1:42" s="99" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:42" s="99" customFormat="1" ht="15" customHeight="1">
       <c r="A65" s="92">
         <v>3</v>
       </c>
       <c r="B65" s="93" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C65" s="100"/>
       <c r="D65" s="95"/>
@@ -9530,12 +9545,12 @@
       <c r="AL65" s="95"/>
       <c r="AM65" s="98"/>
     </row>
-    <row r="66" spans="1:42" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:42" s="142" customFormat="1">
       <c r="A66" s="132">
         <v>3</v>
       </c>
       <c r="B66" s="135" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="C66" s="136">
         <v>45809</v>
@@ -9548,7 +9563,7 @@
         <v>18</v>
       </c>
       <c r="G66" s="138" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="H66" s="138" t="s">
         <v>18</v>
@@ -9645,14 +9660,14 @@
       </c>
       <c r="AM66" s="145"/>
     </row>
-    <row r="67" spans="1:42" s="142" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:42" s="142" customFormat="1">
       <c r="A67" s="147">
         <v>3</v>
       </c>
       <c r="B67" s="148" t="s">
-        <v>101</v>
-      </c>
-      <c r="C67" s="200">
+        <v>114</v>
+      </c>
+      <c r="C67" s="199">
         <v>45870</v>
       </c>
       <c r="D67" s="150"/>
@@ -9705,12 +9720,12 @@
       <c r="AO67" s="147"/>
       <c r="AP67" s="147"/>
     </row>
-    <row r="68" spans="1:42" s="99" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:42" s="99" customFormat="1" ht="17.45" customHeight="1">
       <c r="A68" s="92">
         <v>3</v>
       </c>
       <c r="B68" s="93" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C68" s="100">
         <v>46023</v>
@@ -9766,788 +9781,697 @@
       </c>
       <c r="AM68" s="98"/>
     </row>
-    <row r="70" spans="1:42" s="147" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="155">
+    <row r="69" spans="1:42" s="120" customFormat="1">
+      <c r="A69" s="120">
+        <v>3</v>
+      </c>
+      <c r="B69" s="121" t="s">
+        <v>116</v>
+      </c>
+      <c r="C69" s="209">
+        <v>46357</v>
+      </c>
+      <c r="D69" s="120" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH69" s="210"/>
+      <c r="AI69" s="211"/>
+    </row>
+    <row r="70" spans="1:42">
+      <c r="AH70" s="18"/>
+      <c r="AI70" s="110"/>
+    </row>
+    <row r="71" spans="1:42" s="147" customFormat="1">
+      <c r="A71" s="155">
         <v>2</v>
       </c>
-      <c r="B70" s="156" t="s">
-        <v>105</v>
-      </c>
-      <c r="C70" s="157">
+      <c r="B71" s="156" t="s">
+        <v>118</v>
+      </c>
+      <c r="C71" s="157">
         <v>46082</v>
       </c>
-      <c r="D70" s="158"/>
-      <c r="E70" s="142" t="s">
+      <c r="D71" s="158"/>
+      <c r="E71" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="F70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="G70" s="159" t="s">
-        <v>106</v>
-      </c>
-      <c r="H70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="I70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="J70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="K70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="L70" s="145" t="s">
-        <v>18</v>
-      </c>
-      <c r="M70" s="142" t="s">
+      <c r="F71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="G71" s="159" t="s">
+        <v>119</v>
+      </c>
+      <c r="H71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="I71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="J71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="K71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="L71" s="145" t="s">
+        <v>18</v>
+      </c>
+      <c r="M71" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="N70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="O70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="P70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="R70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="S70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="T70" s="145" t="s">
-        <v>18</v>
-      </c>
-      <c r="U70" s="142" t="s">
+      <c r="N71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="O71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="P71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="R71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="S71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="T71" s="145" t="s">
+        <v>18</v>
+      </c>
+      <c r="U71" s="142" t="s">
         <v>13</v>
       </c>
-      <c r="V70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="W70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="X70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB70" s="145" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC70" s="142" t="s">
+      <c r="V71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="W71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="X71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB71" s="145" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC71" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="AD70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="AE70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="AF70" s="159" t="s">
-        <v>18</v>
-      </c>
-      <c r="AG70" s="159" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH70" s="145" t="s">
-        <v>18</v>
-      </c>
-      <c r="AI70" s="160" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ70" s="161" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK70" s="162" t="s">
+      <c r="AD71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="AE71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF71" s="159" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG71" s="159" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH71" s="145" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI71" s="160" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ71" s="161" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK71" s="162" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:42" s="107" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="102">
+    <row r="72" spans="1:42" s="107" customFormat="1">
+      <c r="A72" s="102">
         <v>2</v>
       </c>
-      <c r="B71" s="103" t="s">
-        <v>107</v>
-      </c>
-      <c r="C71" s="108">
+      <c r="B72" s="103" t="s">
+        <v>120</v>
+      </c>
+      <c r="C72" s="108">
         <v>47027</v>
       </c>
-      <c r="D71" s="104"/>
-      <c r="E71" s="107" t="s">
+      <c r="D72" s="104"/>
+      <c r="E72" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="F71" s="105" t="s">
-        <v>21</v>
-      </c>
-      <c r="G71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="H71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="I71" s="102" t="s">
-        <v>108</v>
-      </c>
-      <c r="J71" s="102" t="s">
+      <c r="F72" s="105" t="s">
+        <v>21</v>
+      </c>
+      <c r="G72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="H72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="I72" s="102" t="s">
+        <v>121</v>
+      </c>
+      <c r="J72" s="102" t="s">
         <v>36</v>
       </c>
-      <c r="K71" s="102" t="s">
+      <c r="K72" s="102" t="s">
         <v>36</v>
       </c>
-      <c r="L71" s="106" t="s">
+      <c r="L72" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="M71" s="107" t="s">
+      <c r="M72" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="N71" s="105" t="s">
-        <v>18</v>
-      </c>
-      <c r="O71" s="102" t="s">
-        <v>18</v>
-      </c>
-      <c r="P71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q71" s="102" t="s">
-        <v>108</v>
-      </c>
-      <c r="R71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="S71" s="102" t="s">
-        <v>18</v>
-      </c>
-      <c r="T71" s="106" t="s">
-        <v>18</v>
-      </c>
-      <c r="U71" s="107" t="s">
+      <c r="N72" s="105" t="s">
+        <v>18</v>
+      </c>
+      <c r="O72" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="P72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q72" s="102" t="s">
+        <v>121</v>
+      </c>
+      <c r="R72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="S72" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="T72" s="106" t="s">
+        <v>18</v>
+      </c>
+      <c r="U72" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="V71" s="105" t="s">
-        <v>21</v>
-      </c>
-      <c r="W71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="X71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y71" s="102" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA71" s="102" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB71" s="106" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC71" s="107" t="s">
+      <c r="V72" s="105" t="s">
+        <v>21</v>
+      </c>
+      <c r="W72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="X72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y72" s="102" t="s">
+        <v>121</v>
+      </c>
+      <c r="Z72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA72" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB72" s="106" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC72" s="107" t="s">
         <v>14</v>
       </c>
-      <c r="AD71" s="105" t="s">
-        <v>21</v>
-      </c>
-      <c r="AE71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="AF71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG71" s="102" t="s">
-        <v>108</v>
-      </c>
-      <c r="AH71" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="AI71" s="102" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ71" s="102" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK71" s="11" t="s">
+      <c r="AD72" s="105" t="s">
+        <v>21</v>
+      </c>
+      <c r="AE72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG72" s="102" t="s">
+        <v>121</v>
+      </c>
+      <c r="AH72" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI72" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ72" s="102" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK72" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="72" spans="1:42" s="142" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="163">
+    <row r="73" spans="1:42" s="142" customFormat="1">
+      <c r="A73" s="163">
         <v>2</v>
       </c>
-      <c r="B72" s="148" t="s">
-        <v>109</v>
-      </c>
-      <c r="C72" s="200">
+      <c r="B73" s="148" t="s">
+        <v>122</v>
+      </c>
+      <c r="C73" s="199">
         <v>46113</v>
       </c>
-      <c r="D72" s="164"/>
-      <c r="E72" s="142" t="s">
-        <v>4</v>
-      </c>
-      <c r="F72" s="165" t="s">
-        <v>21</v>
-      </c>
-      <c r="G72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="H72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="I72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="J72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="K72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="L72" s="150" t="s">
-        <v>18</v>
-      </c>
-      <c r="M72" s="142" t="s">
-        <v>12</v>
-      </c>
-      <c r="N72" s="151" t="s">
-        <v>21</v>
-      </c>
-      <c r="O72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="P72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="R72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="S72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="T72" s="150" t="s">
-        <v>18</v>
-      </c>
-      <c r="U72" s="142" t="s">
-        <v>13</v>
-      </c>
-      <c r="V72" s="151" t="s">
-        <v>21</v>
-      </c>
-      <c r="W72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="X72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB72" s="150" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC72" s="142" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD72" s="151" t="s">
-        <v>18</v>
-      </c>
-      <c r="AE72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="AF72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH72" s="149" t="s">
-        <v>21</v>
-      </c>
-      <c r="AI72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ72" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK72" s="152" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="73" spans="1:42" s="147" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="147">
-        <v>2</v>
-      </c>
-      <c r="B73" s="166" t="s">
-        <v>110</v>
-      </c>
-      <c r="C73" s="167">
-        <v>46143</v>
-      </c>
+      <c r="D73" s="164"/>
       <c r="E73" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="F73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="G73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="H73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="I73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="J73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="K73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="L73" s="147" t="s">
+      <c r="F73" s="165" t="s">
+        <v>21</v>
+      </c>
+      <c r="G73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="H73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="I73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="J73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="K73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="L73" s="150" t="s">
         <v>18</v>
       </c>
       <c r="M73" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="N73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="O73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="P73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="R73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="S73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="T73" s="147" t="s">
+      <c r="N73" s="151" t="s">
+        <v>21</v>
+      </c>
+      <c r="O73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="P73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="R73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="S73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="T73" s="150" t="s">
         <v>18</v>
       </c>
       <c r="U73" s="142" t="s">
         <v>13</v>
       </c>
-      <c r="V73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="W73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="X73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB73" s="147" t="s">
+      <c r="V73" s="151" t="s">
+        <v>21</v>
+      </c>
+      <c r="W73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="X73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB73" s="150" t="s">
         <v>18</v>
       </c>
       <c r="AC73" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="AD73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="AE73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="AF73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="AG73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH73" s="147" t="s">
-        <v>21</v>
-      </c>
-      <c r="AI73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ73" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK73" s="168" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL73" s="169" t="s">
-        <v>23</v>
-      </c>
-      <c r="AM73" s="169"/>
+      <c r="AD73" s="151" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH73" s="149" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ73" s="149" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK73" s="152" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="74" spans="1:42" s="170" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="170">
+    <row r="74" spans="1:42" s="147" customFormat="1">
+      <c r="A74" s="147">
         <v>2</v>
       </c>
-      <c r="B74" s="171" t="s">
-        <v>111</v>
-      </c>
-      <c r="C74" s="172">
-        <v>45901</v>
-      </c>
-      <c r="D74" s="173"/>
+      <c r="B74" s="166" t="s">
+        <v>123</v>
+      </c>
+      <c r="C74" s="167">
+        <v>46143</v>
+      </c>
       <c r="E74" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="F74" s="174" t="s">
-        <v>27</v>
-      </c>
-      <c r="G74" s="170" t="s">
-        <v>28</v>
-      </c>
-      <c r="H74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="I74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="J74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="K74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="L74" s="173" t="s">
+      <c r="F74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="G74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="H74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="I74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="J74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="K74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="L74" s="147" t="s">
         <v>18</v>
       </c>
       <c r="M74" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="N74" s="174" t="s">
-        <v>27</v>
-      </c>
-      <c r="O74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="P74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="R74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="S74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="T74" s="173" t="s">
+      <c r="N74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="O74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="P74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="R74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="S74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="T74" s="147" t="s">
         <v>18</v>
       </c>
       <c r="U74" s="142" t="s">
         <v>13</v>
       </c>
-      <c r="V74" s="174" t="s">
-        <v>27</v>
-      </c>
-      <c r="W74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="X74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="Z74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB74" s="173" t="s">
+      <c r="V74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="W74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="X74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB74" s="147" t="s">
         <v>18</v>
       </c>
       <c r="AC74" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="AD74" s="174" t="s">
-        <v>27</v>
-      </c>
-      <c r="AE74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AF74" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AG74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AH74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AI74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AJ74" s="170" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK74" s="175" t="s">
+      <c r="AD74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="AE74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH74" s="147" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ74" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK74" s="168" t="s">
         <v>39</v>
       </c>
+      <c r="AL74" s="169" t="s">
+        <v>23</v>
+      </c>
+      <c r="AM74" s="169"/>
     </row>
-    <row r="75" spans="1:42" s="142" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="142">
+    <row r="75" spans="1:42" s="170" customFormat="1">
+      <c r="A75" s="170">
         <v>2</v>
       </c>
-      <c r="B75" s="166" t="s">
-        <v>112</v>
-      </c>
-      <c r="C75" s="167">
-        <v>46113</v>
-      </c>
-      <c r="D75" s="147"/>
+      <c r="B75" s="171" t="s">
+        <v>124</v>
+      </c>
+      <c r="C75" s="172">
+        <v>45901</v>
+      </c>
+      <c r="D75" s="173"/>
       <c r="E75" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="F75" s="147"/>
-      <c r="G75" s="147"/>
-      <c r="H75" s="147"/>
-      <c r="I75" s="147"/>
-      <c r="J75" s="147"/>
-      <c r="K75" s="147"/>
-      <c r="L75" s="147"/>
+      <c r="F75" s="174" t="s">
+        <v>27</v>
+      </c>
+      <c r="G75" s="170" t="s">
+        <v>28</v>
+      </c>
+      <c r="H75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="I75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="J75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="K75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="L75" s="173" t="s">
+        <v>18</v>
+      </c>
       <c r="M75" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="N75" s="147"/>
-      <c r="O75" s="147"/>
-      <c r="P75" s="147"/>
-      <c r="Q75" s="147"/>
-      <c r="R75" s="147"/>
-      <c r="S75" s="147"/>
-      <c r="T75" s="147"/>
+      <c r="N75" s="174" t="s">
+        <v>27</v>
+      </c>
+      <c r="O75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="P75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="R75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="S75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="T75" s="173" t="s">
+        <v>18</v>
+      </c>
       <c r="U75" s="142" t="s">
         <v>13</v>
       </c>
-      <c r="V75" s="147"/>
-      <c r="W75" s="147"/>
-      <c r="X75" s="147"/>
-      <c r="Y75" s="147"/>
-      <c r="Z75" s="147"/>
-      <c r="AA75" s="147"/>
-      <c r="AB75" s="147"/>
+      <c r="V75" s="174" t="s">
+        <v>27</v>
+      </c>
+      <c r="W75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="X75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB75" s="173" t="s">
+        <v>18</v>
+      </c>
       <c r="AC75" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="AD75" s="147"/>
-      <c r="AE75" s="147"/>
-      <c r="AF75" s="147"/>
-      <c r="AG75" s="147"/>
-      <c r="AH75" s="147"/>
-      <c r="AI75" s="147"/>
-      <c r="AJ75" s="147"/>
-      <c r="AK75" s="162" t="s">
+      <c r="AD75" s="174" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AF75" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AG75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ75" s="170" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK75" s="175" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="79" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="B79" s="154" t="s">
-        <v>132</v>
+    <row r="76" spans="1:42" s="142" customFormat="1">
+      <c r="A76" s="142">
+        <v>2</v>
+      </c>
+      <c r="B76" s="166" t="s">
+        <v>125</v>
+      </c>
+      <c r="C76" s="167">
+        <v>46113</v>
+      </c>
+      <c r="D76" s="147"/>
+      <c r="E76" s="142" t="s">
+        <v>4</v>
+      </c>
+      <c r="F76" s="147"/>
+      <c r="G76" s="147"/>
+      <c r="H76" s="147"/>
+      <c r="I76" s="147"/>
+      <c r="J76" s="147"/>
+      <c r="K76" s="147"/>
+      <c r="L76" s="147"/>
+      <c r="M76" s="142" t="s">
+        <v>12</v>
+      </c>
+      <c r="N76" s="147"/>
+      <c r="O76" s="147"/>
+      <c r="P76" s="147"/>
+      <c r="Q76" s="147"/>
+      <c r="R76" s="147"/>
+      <c r="S76" s="147"/>
+      <c r="T76" s="147"/>
+      <c r="U76" s="142" t="s">
+        <v>13</v>
+      </c>
+      <c r="V76" s="147"/>
+      <c r="W76" s="147"/>
+      <c r="X76" s="147"/>
+      <c r="Y76" s="147"/>
+      <c r="Z76" s="147"/>
+      <c r="AA76" s="147"/>
+      <c r="AB76" s="147"/>
+      <c r="AC76" s="142" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD76" s="147"/>
+      <c r="AE76" s="147"/>
+      <c r="AF76" s="147"/>
+      <c r="AG76" s="147"/>
+      <c r="AH76" s="147"/>
+      <c r="AI76" s="147"/>
+      <c r="AJ76" s="147"/>
+      <c r="AK76" s="162" t="s">
+        <v>39</v>
       </c>
     </row>
-    <row r="80" spans="1:42" s="153" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="41">
+    <row r="80" spans="1:42">
+      <c r="B80" s="154" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="81" spans="1:39" s="153" customFormat="1">
+      <c r="A81" s="41">
         <v>3</v>
       </c>
-      <c r="B80" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="C80" s="43">
+      <c r="B81" s="42" t="s">
+        <v>127</v>
+      </c>
+      <c r="C81" s="43">
         <v>45901</v>
       </c>
-      <c r="D80" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="E80" s="49" t="s">
-        <v>4</v>
-      </c>
-      <c r="F80" s="45"/>
-      <c r="G80" s="45"/>
-      <c r="H80" s="45"/>
-      <c r="I80" s="45"/>
-      <c r="J80" s="45"/>
-      <c r="K80" s="45"/>
-      <c r="L80" s="44"/>
-      <c r="M80" s="49" t="s">
-        <v>12</v>
-      </c>
-      <c r="N80" s="45"/>
-      <c r="O80" s="45"/>
-      <c r="P80" s="45"/>
-      <c r="Q80" s="45"/>
-      <c r="R80" s="45"/>
-      <c r="S80" s="45"/>
-      <c r="T80" s="44"/>
-      <c r="U80" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="V80" s="45"/>
-      <c r="W80" s="45"/>
-      <c r="X80" s="45"/>
-      <c r="Y80" s="45"/>
-      <c r="Z80" s="45"/>
-      <c r="AA80" s="45"/>
-      <c r="AB80" s="44"/>
-      <c r="AC80" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD80" s="45"/>
-      <c r="AE80" s="45"/>
-      <c r="AF80" s="45"/>
-      <c r="AG80" s="45"/>
-      <c r="AH80" s="44"/>
-      <c r="AI80" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="AJ80" s="47" t="s">
-        <v>27</v>
-      </c>
-      <c r="AK80" s="45">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="81" spans="1:39" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="41">
-        <v>6</v>
-      </c>
-      <c r="B81" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="C81" s="43">
-        <v>44621</v>
-      </c>
-      <c r="D81" s="44"/>
+      <c r="D81" s="44" t="s">
+        <v>128</v>
+      </c>
       <c r="E81" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="F81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="G81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="H81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="I81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="J81" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="K81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="L81" s="44" t="s">
-        <v>27</v>
-      </c>
+      <c r="F81" s="45"/>
+      <c r="G81" s="45"/>
+      <c r="H81" s="45"/>
+      <c r="I81" s="45"/>
+      <c r="J81" s="45"/>
+      <c r="K81" s="45"/>
+      <c r="L81" s="44"/>
       <c r="M81" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="N81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="O81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="P81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="R81" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="S81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="T81" s="44" t="s">
-        <v>27</v>
-      </c>
+      <c r="N81" s="45"/>
+      <c r="O81" s="45"/>
+      <c r="P81" s="45"/>
+      <c r="Q81" s="45"/>
+      <c r="R81" s="45"/>
+      <c r="S81" s="45"/>
+      <c r="T81" s="44"/>
       <c r="U81" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="V81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="W81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="X81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z81" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB81" s="44" t="s">
-        <v>27</v>
-      </c>
+      <c r="V81" s="45"/>
+      <c r="W81" s="45"/>
+      <c r="X81" s="45"/>
+      <c r="Y81" s="45"/>
+      <c r="Z81" s="45"/>
+      <c r="AA81" s="45"/>
+      <c r="AB81" s="44"/>
       <c r="AC81" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="AD81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="AE81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF81" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="AG81" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="AH81" s="44" t="s">
-        <v>27</v>
-      </c>
+      <c r="AD81" s="45"/>
+      <c r="AE81" s="45"/>
+      <c r="AF81" s="45"/>
+      <c r="AG81" s="45"/>
+      <c r="AH81" s="44"/>
       <c r="AI81" s="46" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="AJ81" s="47" t="s">
         <v>27</v>
@@ -10555,29 +10479,140 @@
       <c r="AK81" s="45">
         <v>37.5</v>
       </c>
-      <c r="AL81" s="44" t="s">
+    </row>
+    <row r="82" spans="1:39" s="49" customFormat="1">
+      <c r="A82" s="41">
+        <v>6</v>
+      </c>
+      <c r="B82" s="42" t="s">
+        <v>129</v>
+      </c>
+      <c r="C82" s="43">
+        <v>44621</v>
+      </c>
+      <c r="D82" s="44"/>
+      <c r="E82" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="H82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="I82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="J82" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="K82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="L82" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="M82" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="N82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="O82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="P82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="R82" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="S82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="T82" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="U82" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="V82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="W82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="X82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z82" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB82" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC82" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF82" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG82" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="AH82" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="AI82" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ82" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="AK82" s="45">
+        <v>37.5</v>
+      </c>
+      <c r="AL82" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="AM81" s="48"/>
+      <c r="AM82" s="48"/>
     </row>
-    <row r="85" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="B85" s="143" t="s">
-        <v>118</v>
+    <row r="86" spans="1:39">
+      <c r="B86" s="143" t="s">
+        <v>130</v>
       </c>
     </row>
-    <row r="87" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="B87" s="146" t="s">
-        <v>116</v>
+    <row r="88" spans="1:39">
+      <c r="B88" s="146" t="s">
+        <v>131</v>
       </c>
     </row>
-    <row r="89" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="B89" s="121" t="s">
-        <v>120</v>
+    <row r="90" spans="1:39">
+      <c r="B90" s="121" t="s">
+        <v>132</v>
       </c>
     </row>
-    <row r="91" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="B91" s="131" t="s">
-        <v>114</v>
+    <row r="92" spans="1:39">
+      <c r="B92" s="131" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>